<commit_message>
calibrated electricity demand water
</commit_message>
<xml_diff>
--- a/ssp_modeling/input_data/reference/Libya_Water_Energy_Model_2020-2050-v6_final_cleanup.xlsx
+++ b/ssp_modeling/input_data/reference/Libya_Water_Energy_Model_2020-2050-v6_final_cleanup.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fabianfuentes/git/ssp_libya/ssp_modeling/input_data/reference/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5313CD7F-2899-2F4E-9928-8A3D165677B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C84F52E8-A899-7A4A-9A59-6294E73CFBB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-51200" yWindow="-7160" windowWidth="25600" windowHeight="28200" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-51200" yWindow="-7160" windowWidth="51200" windowHeight="28200" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,20 @@
     <sheet name="Energy" sheetId="5" r:id="rId5"/>
     <sheet name="Summary" sheetId="6" r:id="rId6"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlchart.v1.0" hidden="1">Energy!$A$19:$C$19</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">Energy!$A$20:$C$20</definedName>
+    <definedName name="_xlchart.v1.10" hidden="1">Energy!$D$20:$AH$20</definedName>
+    <definedName name="_xlchart.v1.11" hidden="1">Energy!$D$21:$AH$21</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">Energy!$A$21:$C$21</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">Energy!$D$19:$AH$19</definedName>
+    <definedName name="_xlchart.v1.4" hidden="1">Energy!$D$20:$AH$20</definedName>
+    <definedName name="_xlchart.v1.5" hidden="1">Energy!$D$21:$AH$21</definedName>
+    <definedName name="_xlchart.v1.6" hidden="1">Energy!$A$19:$C$19</definedName>
+    <definedName name="_xlchart.v1.7" hidden="1">Energy!$A$20:$C$20</definedName>
+    <definedName name="_xlchart.v1.8" hidden="1">Energy!$A$21:$C$21</definedName>
+    <definedName name="_xlchart.v1.9" hidden="1">Energy!$D$19:$AH$19</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -1043,7 +1057,7 @@
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="0.000"/>
   </numFmts>
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1156,8 +1170,15 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1229,12 +1250,6 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="3" tint="0.59999389629810485"/>
-        <bgColor rgb="FFE4F6E1"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -1260,10 +1275,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1355,15 +1371,17 @@
     <xf numFmtId="2" fontId="12" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="2" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="2" fontId="12" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1447,6 +1465,674 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-MX"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Energy!$A$19:$C$19</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>BAU</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>PJ/yr</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>GW + GMMR + RW</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Energy!$D$19:$AH$19</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="31"/>
+                <c:pt idx="0">
+                  <c:v>28.025346321149403</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>28.017108786942355</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>28.007264140696478</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>27.995824689483172</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>27.982802730808359</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>27.968210551721373</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>27.952060427938289</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>27.93436462297981</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>27.774753560067115</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>27.122502611699357</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>26.474019149026752</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>25.829305071206161</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>25.188363417837991</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>24.551198343389132</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>23.917815091976731</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>23.288219972508841</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>22.662420334177948</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>22.67442954230329</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>22.683681954518111</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>22.690187897298028</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>22.693958642826427</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>22.695006386193327</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>22.693344222923784</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>22.688986126832006</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>22.681946928197757</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>22.672242292261053</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>22.65988869803169</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>22.644903417410013</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>22.627304494615302</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>22.607110725918147</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>22.584341639673617</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-5DFD-6545-A6F5-826853920347}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Energy!$A$20:$C$20</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>Unconditional</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>PJ/yr</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>GW + GMMR + RW + DESAL</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Energy!$D$20:$AH$20</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="31"/>
+                <c:pt idx="0">
+                  <c:v>28.025346321149403</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>28.017108786942355</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>28.007264140696478</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>27.995824689483172</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>27.982802730808359</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>27.968210551721373</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>27.952060427938289</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>27.93436462297981</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>28.055517214579371</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>28.666267303437827</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>29.270231962210435</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>29.867433704538762</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>30.457893871028471</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>31.041632653267975</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>31.618669117512773</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>32.189021228039195</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>32.75270587017129</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>32.675733872984466</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>32.598695031689616</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>32.521603129701276</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>32.444470960393318</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>32.367310348545999</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>32.290132171487343</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>32.212946379932959</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>32.135762018527103</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>32.058587246088912</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>31.981429355566831</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>31.904294793704651</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>31.827189180422515</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>31.750117327916154</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>31.673083259477465</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-5DFD-6545-A6F5-826853920347}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Energy!$A$21:$C$21</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>Conditional</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>PJ/yr</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>GW + GMMR + RW + DESAL</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Energy!$D$21:$AH$21</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="31"/>
+                <c:pt idx="0">
+                  <c:v>28.025346321149403</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>28.017108786942355</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>28.007264140696478</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>27.995824689483172</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>27.982802730808359</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>27.968210551721373</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>27.952060427938289</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>27.93436462297981</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>28.055517214579371</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>28.666267303437827</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>29.270231962210435</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>29.867433704538762</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>30.457893871028471</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>31.041632653267975</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>31.618669117512773</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>32.189021228039195</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>32.75270587017129</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>32.675733872984466</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>32.598695031689616</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>32.521603129701276</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>32.444470960393318</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>32.367310348545999</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>32.290132171487343</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>32.212946379932959</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>32.135762018527103</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>32.058587246088912</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>31.981429355566831</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>31.904294793704651</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>31.827189180422515</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>31.750117327916154</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>31.673083259477465</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-5DFD-6545-A6F5-826853920347}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:smooth val="0"/>
+        <c:axId val="1749678976"/>
+        <c:axId val="1749666880"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="1749678976"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-MX"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1749666880"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1749666880"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-MX"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1749678976"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-MX"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-MX"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -2498,7 +3184,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -3779,7 +4465,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -4831,7 +5517,604 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>310029</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>136525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>420220</xdr:colOff>
+      <xdr:row>57</xdr:row>
+      <xdr:rowOff>140073</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{591364D0-C824-B88F-76A5-044B49745FA2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor>
     <xdr:from>
@@ -12295,7 +13578,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:AH25"/>
+  <dimension ref="A1:AI29"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="36" customWidth="1"/>
@@ -13234,128 +14517,128 @@
         <v>308</v>
       </c>
       <c r="D12" s="22">
-        <f>D7*Supply!D14</f>
-        <v>17122.589571324999</v>
+        <f>D7*Supply!D31</f>
+        <v>0</v>
       </c>
       <c r="E12" s="22">
-        <f>E7*Supply!E14</f>
-        <v>17116.000527355784</v>
+        <f>E7*Supply!E31</f>
+        <v>0</v>
       </c>
       <c r="F12" s="22">
-        <f>F7*Supply!F14</f>
-        <v>17106.415461208257</v>
+        <f>F7*Supply!F31</f>
+        <v>0</v>
       </c>
       <c r="G12" s="22">
-        <f>G7*Supply!G14</f>
-        <v>17093.898775745289</v>
+        <f>G7*Supply!G31</f>
+        <v>0</v>
       </c>
       <c r="H12" s="22">
-        <f>H7*Supply!H14</f>
-        <v>17078.513906770877</v>
+        <f>H7*Supply!H31</f>
+        <v>0</v>
       </c>
       <c r="I12" s="22">
-        <f>I7*Supply!I14</f>
-        <v>17060.323335408189</v>
+        <f>I7*Supply!I31</f>
+        <v>0</v>
       </c>
       <c r="J12" s="22">
-        <f>J7*Supply!J14</f>
-        <v>17039.388600333219</v>
+        <f>J7*Supply!J31</f>
+        <v>0</v>
       </c>
       <c r="K12" s="22">
-        <f>K7*Supply!K14</f>
-        <v>17015.770309865635</v>
+        <f>K7*Supply!K31</f>
+        <v>0</v>
       </c>
       <c r="L12" s="22">
-        <f>L7*Supply!L14</f>
-        <v>16989.528153918447</v>
+        <f>L7*Supply!L31</f>
+        <v>38.994952015591252</v>
       </c>
       <c r="M12" s="22">
-        <f>M7*Supply!M14</f>
-        <v>16960.720915807982</v>
+        <f>M7*Supply!M31</f>
+        <v>214.41176274145431</v>
       </c>
       <c r="N12" s="22">
-        <f>N7*Supply!N14</f>
-        <v>16929.406483925683</v>
+        <f>N7*Supply!N31</f>
+        <v>388.36289071995606</v>
       </c>
       <c r="O12" s="22">
-        <f>O7*Supply!O14</f>
-        <v>16895.641863273395</v>
+        <f>O7*Supply!O31</f>
+        <v>560.85119907397268</v>
       </c>
       <c r="P12" s="22">
-        <f>P7*Supply!P14</f>
-        <v>16859.483186863406</v>
+        <f>P7*Supply!P31</f>
+        <v>731.87922960978881</v>
       </c>
       <c r="Q12" s="22">
-        <f>Q7*Supply!Q14</f>
-        <v>16820.985726984934</v>
+        <f>Q7*Supply!Q31</f>
+        <v>901.44920970539511</v>
       </c>
       <c r="R12" s="22">
-        <f>R7*Supply!R14</f>
-        <v>16780.203906338476</v>
+        <f>R7*Supply!R31</f>
+        <v>1069.5630591022277</v>
       </c>
       <c r="S12" s="22">
-        <f>S7*Supply!S14</f>
-        <v>16737.191309039357</v>
+        <f>S7*Supply!S31</f>
+        <v>1236.222396601438</v>
       </c>
       <c r="T12" s="22">
-        <f>T7*Supply!T14</f>
-        <v>16692.000691492121</v>
+        <f>T7*Supply!T31</f>
+        <v>1401.4285466657416</v>
       </c>
       <c r="U12" s="22">
-        <f>U7*Supply!U14</f>
-        <v>16644.683993137001</v>
+        <f>U7*Supply!U31</f>
+        <v>1389.0700459279419</v>
       </c>
       <c r="V12" s="22">
-        <f>V7*Supply!V14</f>
-        <v>16595.292347069997</v>
+        <f>V7*Supply!V31</f>
+        <v>1377.0851496071541</v>
       </c>
       <c r="W12" s="22">
-        <f>W7*Supply!W14</f>
-        <v>16543.876090537939</v>
+        <f>W7*Supply!W31</f>
+        <v>1365.4743378337839</v>
       </c>
       <c r="X12" s="22">
-        <f>X7*Supply!X14</f>
-        <v>16490.484775309815</v>
+        <f>X7*Supply!X31</f>
+        <v>1354.237821884291</v>
       </c>
       <c r="Y12" s="22">
-        <f>Y7*Supply!Y14</f>
-        <v>16435.167177925916</v>
+        <f>Y7*Supply!Y31</f>
+        <v>1343.3755503267594</v>
       </c>
       <c r="Z12" s="22">
-        <f>Z7*Supply!Z14</f>
-        <v>16377.971309825931</v>
+        <f>Z7*Supply!Z31</f>
+        <v>1332.8872150782729</v>
       </c>
       <c r="AA12" s="22">
-        <f>AA7*Supply!AA14</f>
-        <v>16318.944427357555</v>
+        <f>AA7*Supply!AA31</f>
+        <v>1322.7722573751323</v>
       </c>
       <c r="AB12" s="22">
-        <f>AB7*Supply!AB14</f>
-        <v>16258.133041666701</v>
+        <f>AB7*Supply!AB31</f>
+        <v>1313.0298736568536</v>
       </c>
       <c r="AC12" s="22">
-        <f>AC7*Supply!AC14</f>
-        <v>16195.582928470825</v>
+        <f>AC7*Supply!AC31</f>
+        <v>1303.6590213649808</v>
       </c>
       <c r="AD12" s="22">
-        <f>AD7*Supply!AD14</f>
-        <v>16131.33913771657</v>
+        <f>AD7*Supply!AD31</f>
+        <v>1294.6584246576592</v>
       </c>
       <c r="AE12" s="22">
-        <f>AE7*Supply!AE14</f>
-        <v>16065.446003122936</v>
+        <f>AE7*Supply!AE31</f>
+        <v>1286.0265800409222</v>
       </c>
       <c r="AF12" s="22">
-        <f>AF7*Supply!AF14</f>
-        <v>15997.947151611452</v>
+        <f>AF7*Supply!AF31</f>
+        <v>1277.7617619176688</v>
       </c>
       <c r="AG12" s="22">
-        <f>AG7*Supply!AG14</f>
-        <v>15928.885512624334</v>
+        <f>AG7*Supply!AG31</f>
+        <v>1269.8620280552782</v>
       </c>
       <c r="AH12" s="22">
-        <f>AH7*Supply!AH14</f>
-        <v>15858.303327332134</v>
+        <f>AH7*Supply!AH31</f>
+        <v>1262.3252249727561</v>
       </c>
     </row>
     <row r="13" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -13898,7 +15181,7 @@
         <v>7.5357534582154289</v>
       </c>
     </row>
-    <row r="17" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="23"/>
       <c r="B17" s="58" t="s">
         <v>322</v>
@@ -14031,7 +15314,7 @@
         <v>27.128712449575541</v>
       </c>
     </row>
-    <row r="18" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="23"/>
       <c r="B18" s="14"/>
       <c r="C18" s="15"/>
@@ -14067,7 +15350,7 @@
       <c r="AG18" s="65"/>
       <c r="AH18" s="65"/>
     </row>
-    <row r="19" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="63" t="s">
         <v>324</v>
       </c>
@@ -14078,131 +15361,131 @@
         <v>328</v>
       </c>
       <c r="D19" s="64">
-        <f>+(D9+D10+D14)* 0.0036</f>
-        <v>15.170497668104401</v>
+        <f>+(D9+D10+(D11-D12)+D14)* 0.0036</f>
+        <v>28.025346321149403</v>
       </c>
       <c r="E19" s="64">
-        <f t="shared" ref="E19:AH19" si="3">+(E9+E10+E14)* 0.0036</f>
-        <v>15.1283462930565</v>
+        <f t="shared" ref="E19:AH19" si="3">+(E9+E10+(E11-E12)+E14)* 0.0036</f>
+        <v>28.017108786942355</v>
       </c>
       <c r="F19" s="64">
         <f t="shared" si="3"/>
-        <v>15.086763149119758</v>
+        <v>28.007264140696478</v>
       </c>
       <c r="G19" s="64">
         <f t="shared" si="3"/>
-        <v>15.045732063612462</v>
+        <v>27.995824689483172</v>
       </c>
       <c r="H19" s="64">
         <f t="shared" si="3"/>
-        <v>15.00523712257224</v>
+        <v>27.982802730808359</v>
       </c>
       <c r="I19" s="64">
         <f t="shared" si="3"/>
-        <v>14.965262667704668</v>
+        <v>27.968210551721373</v>
       </c>
       <c r="J19" s="64">
         <f t="shared" si="3"/>
-        <v>14.925793293362332</v>
+        <v>27.952060427938289</v>
       </c>
       <c r="K19" s="64">
         <f t="shared" si="3"/>
-        <v>14.886813843553981</v>
+        <v>27.93436462297981</v>
       </c>
       <c r="L19" s="64">
         <f t="shared" si="3"/>
-        <v>14.848309408983555</v>
+        <v>27.774753560067115</v>
       </c>
       <c r="M19" s="64">
         <f t="shared" si="3"/>
-        <v>14.810265324118784</v>
+        <v>27.122502611699357</v>
       </c>
       <c r="N19" s="64">
         <f t="shared" si="3"/>
-        <v>14.772667164289111</v>
+        <v>26.474019149026752</v>
       </c>
       <c r="O19" s="64">
         <f t="shared" si="3"/>
-        <v>14.735500742812677</v>
+        <v>25.829305071206161</v>
       </c>
       <c r="P19" s="64">
         <f t="shared" si="3"/>
-        <v>14.698752108152071</v>
+        <v>25.188363417837991</v>
       </c>
       <c r="Q19" s="64">
         <f t="shared" si="3"/>
-        <v>14.662407541098633</v>
+        <v>24.551198343389132</v>
       </c>
       <c r="R19" s="64">
         <f t="shared" si="3"/>
-        <v>14.626453551985021</v>
+        <v>23.917815091976731</v>
       </c>
       <c r="S19" s="64">
         <f t="shared" si="3"/>
-        <v>14.590876877925789</v>
+        <v>23.288219972508841</v>
       </c>
       <c r="T19" s="64">
         <f t="shared" si="3"/>
-        <v>14.555664480085737</v>
+        <v>22.662420334177948</v>
       </c>
       <c r="U19" s="64">
         <f t="shared" si="3"/>
-        <v>14.520803540975756</v>
+        <v>22.67442954230329</v>
       </c>
       <c r="V19" s="64">
         <f t="shared" si="3"/>
-        <v>14.486281461775947</v>
+        <v>22.683681954518111</v>
       </c>
       <c r="W19" s="64">
         <f t="shared" si="3"/>
-        <v>14.45208585968575</v>
+        <v>22.690187897298028</v>
       </c>
       <c r="X19" s="64">
         <f t="shared" si="3"/>
-        <v>14.418204565300833</v>
+        <v>22.693958642826427</v>
       </c>
       <c r="Y19" s="64">
         <f t="shared" si="3"/>
-        <v>14.38462562001652</v>
+        <v>22.695006386193327</v>
       </c>
       <c r="Z19" s="64">
         <f t="shared" si="3"/>
-        <v>14.351337273457478</v>
+        <v>22.693344222923784</v>
       </c>
       <c r="AA19" s="64">
         <f t="shared" si="3"/>
-        <v>14.318327980933487</v>
+        <v>22.688986126832006</v>
       </c>
       <c r="AB19" s="64">
         <f t="shared" si="3"/>
-        <v>14.285586400920973</v>
+        <v>22.681946928197757</v>
       </c>
       <c r="AC19" s="64">
         <f t="shared" si="3"/>
-        <v>14.253101392570159</v>
+        <v>22.672242292261053</v>
       </c>
       <c r="AD19" s="64">
         <f t="shared" si="3"/>
-        <v>14.220862013237502</v>
+        <v>22.65988869803169</v>
       </c>
       <c r="AE19" s="64">
         <f t="shared" si="3"/>
-        <v>14.188857516043303</v>
+        <v>22.644903417410013</v>
       </c>
       <c r="AF19" s="64">
         <f t="shared" si="3"/>
-        <v>14.157077347454138</v>
+        <v>22.627304494615302</v>
       </c>
       <c r="AG19" s="64">
         <f t="shared" si="3"/>
-        <v>14.125511144889975</v>
+        <v>22.607110725918147</v>
       </c>
       <c r="AH19" s="64">
-        <f t="shared" si="3"/>
-        <v>14.094148734355709</v>
-      </c>
-    </row>
-    <row r="20" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+        <f>+(AH9+AH10+(AH11-AH12)+AH14)* 0.0036</f>
+        <v>22.584341639673617</v>
+      </c>
+    </row>
+    <row r="20" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="63" t="s">
         <v>325</v>
       </c>
@@ -14213,267 +15496,268 @@
         <v>329</v>
       </c>
       <c r="D20" s="64">
-        <f>+(D9+D10+D14)* 0.0036</f>
-        <v>15.170497668104401</v>
+        <f>+(D9+D10+D11+D12+D14)* 0.0036</f>
+        <v>28.025346321149403</v>
       </c>
       <c r="E20" s="64">
-        <f t="shared" ref="E20:H20" si="4">+(E9+E10+E14)* 0.0036</f>
-        <v>15.1283462930565</v>
+        <f t="shared" ref="E20:AH20" si="4">+(E9+E10+E11+E12+E14)* 0.0036</f>
+        <v>28.017108786942355</v>
       </c>
       <c r="F20" s="64">
         <f t="shared" si="4"/>
-        <v>15.086763149119758</v>
+        <v>28.007264140696478</v>
       </c>
       <c r="G20" s="64">
         <f t="shared" si="4"/>
-        <v>15.045732063612462</v>
+        <v>27.995824689483172</v>
       </c>
       <c r="H20" s="64">
         <f t="shared" si="4"/>
-        <v>15.00523712257224</v>
-      </c>
-      <c r="I20" s="67">
-        <f t="shared" ref="I20:AH20" si="5">+(I9+I10+I14+I11)* 0.0036</f>
-        <v>27.96821055172137</v>
-      </c>
-      <c r="J20" s="67">
+        <v>27.982802730808359</v>
+      </c>
+      <c r="I20" s="64">
+        <f t="shared" si="4"/>
+        <v>27.968210551721373</v>
+      </c>
+      <c r="J20" s="64">
+        <f t="shared" si="4"/>
+        <v>27.952060427938289</v>
+      </c>
+      <c r="K20" s="64">
+        <f t="shared" si="4"/>
+        <v>27.93436462297981</v>
+      </c>
+      <c r="L20" s="64">
+        <f t="shared" si="4"/>
+        <v>28.055517214579371</v>
+      </c>
+      <c r="M20" s="64">
+        <f t="shared" si="4"/>
+        <v>28.666267303437827</v>
+      </c>
+      <c r="N20" s="64">
+        <f t="shared" si="4"/>
+        <v>29.270231962210435</v>
+      </c>
+      <c r="O20" s="64">
+        <f t="shared" si="4"/>
+        <v>29.867433704538762</v>
+      </c>
+      <c r="P20" s="64">
+        <f t="shared" si="4"/>
+        <v>30.457893871028471</v>
+      </c>
+      <c r="Q20" s="64">
+        <f t="shared" si="4"/>
+        <v>31.041632653267975</v>
+      </c>
+      <c r="R20" s="64">
+        <f t="shared" si="4"/>
+        <v>31.618669117512773</v>
+      </c>
+      <c r="S20" s="64">
+        <f t="shared" si="4"/>
+        <v>32.189021228039195</v>
+      </c>
+      <c r="T20" s="64">
+        <f t="shared" si="4"/>
+        <v>32.75270587017129</v>
+      </c>
+      <c r="U20" s="64">
+        <f t="shared" si="4"/>
+        <v>32.675733872984466</v>
+      </c>
+      <c r="V20" s="64">
+        <f t="shared" si="4"/>
+        <v>32.598695031689616</v>
+      </c>
+      <c r="W20" s="64">
+        <f t="shared" si="4"/>
+        <v>32.521603129701276</v>
+      </c>
+      <c r="X20" s="64">
+        <f t="shared" si="4"/>
+        <v>32.444470960393318</v>
+      </c>
+      <c r="Y20" s="64">
+        <f t="shared" si="4"/>
+        <v>32.367310348545999</v>
+      </c>
+      <c r="Z20" s="64">
+        <f t="shared" si="4"/>
+        <v>32.290132171487343</v>
+      </c>
+      <c r="AA20" s="64">
+        <f t="shared" si="4"/>
+        <v>32.212946379932959</v>
+      </c>
+      <c r="AB20" s="64">
+        <f t="shared" si="4"/>
+        <v>32.135762018527103</v>
+      </c>
+      <c r="AC20" s="64">
+        <f t="shared" si="4"/>
+        <v>32.058587246088912</v>
+      </c>
+      <c r="AD20" s="64">
+        <f t="shared" si="4"/>
+        <v>31.981429355566831</v>
+      </c>
+      <c r="AE20" s="64">
+        <f t="shared" si="4"/>
+        <v>31.904294793704651</v>
+      </c>
+      <c r="AF20" s="64">
+        <f t="shared" si="4"/>
+        <v>31.827189180422515</v>
+      </c>
+      <c r="AG20" s="64">
+        <f t="shared" si="4"/>
+        <v>31.750117327916154</v>
+      </c>
+      <c r="AH20" s="64">
+        <f t="shared" si="4"/>
+        <v>31.673083259477465</v>
+      </c>
+      <c r="AI20" s="71"/>
+    </row>
+    <row r="21" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="63" t="s">
+        <v>326</v>
+      </c>
+      <c r="B21" s="58" t="s">
+        <v>322</v>
+      </c>
+      <c r="C21" s="62" t="s">
+        <v>329</v>
+      </c>
+      <c r="D21" s="64">
+        <f>+(D9+D10+D11+D12+D14)* 0.0036</f>
+        <v>28.025346321149403</v>
+      </c>
+      <c r="E21" s="64">
+        <f t="shared" ref="E21:AH21" si="5">+(E9+E10+E11+E12+E14)* 0.0036</f>
+        <v>28.017108786942355</v>
+      </c>
+      <c r="F21" s="64">
+        <f t="shared" si="5"/>
+        <v>28.007264140696478</v>
+      </c>
+      <c r="G21" s="64">
+        <f t="shared" si="5"/>
+        <v>27.995824689483172</v>
+      </c>
+      <c r="H21" s="64">
+        <f t="shared" si="5"/>
+        <v>27.982802730808359</v>
+      </c>
+      <c r="I21" s="64">
+        <f t="shared" si="5"/>
+        <v>27.968210551721373</v>
+      </c>
+      <c r="J21" s="64">
         <f t="shared" si="5"/>
         <v>27.952060427938289</v>
       </c>
-      <c r="K20" s="67">
+      <c r="K21" s="64">
         <f t="shared" si="5"/>
-        <v>27.934364622979814</v>
-      </c>
-      <c r="L20" s="67">
+        <v>27.93436462297981</v>
+      </c>
+      <c r="L21" s="64">
         <f t="shared" si="5"/>
-        <v>27.915135387323247</v>
-      </c>
-      <c r="M20" s="67">
+        <v>28.055517214579371</v>
+      </c>
+      <c r="M21" s="64">
         <f t="shared" si="5"/>
-        <v>27.89438495756859</v>
-      </c>
-      <c r="N20" s="67">
+        <v>28.666267303437827</v>
+      </c>
+      <c r="N21" s="64">
         <f t="shared" si="5"/>
-        <v>27.872125555618592</v>
-      </c>
-      <c r="O20" s="67">
+        <v>29.270231962210435</v>
+      </c>
+      <c r="O21" s="64">
         <f t="shared" si="5"/>
-        <v>27.848369387872459</v>
-      </c>
-      <c r="P20" s="67">
+        <v>29.867433704538762</v>
+      </c>
+      <c r="P21" s="64">
         <f t="shared" si="5"/>
-        <v>27.823128644433229</v>
-      </c>
-      <c r="Q20" s="67">
+        <v>30.457893871028471</v>
+      </c>
+      <c r="Q21" s="64">
         <f t="shared" si="5"/>
-        <v>27.796415498328553</v>
-      </c>
-      <c r="R20" s="67">
+        <v>31.041632653267975</v>
+      </c>
+      <c r="R21" s="64">
         <f t="shared" si="5"/>
-        <v>27.768242104744747</v>
-      </c>
-      <c r="S20" s="67">
+        <v>31.618669117512773</v>
+      </c>
+      <c r="S21" s="64">
         <f t="shared" si="5"/>
-        <v>27.738620600274018</v>
-      </c>
-      <c r="T20" s="67">
+        <v>32.189021228039195</v>
+      </c>
+      <c r="T21" s="64">
         <f t="shared" si="5"/>
-        <v>27.707563102174618</v>
-      </c>
-      <c r="U20" s="67">
+        <v>32.75270587017129</v>
+      </c>
+      <c r="U21" s="64">
         <f t="shared" si="5"/>
-        <v>27.67508170764388</v>
-      </c>
-      <c r="V20" s="67">
+        <v>32.675733872984466</v>
+      </c>
+      <c r="V21" s="64">
         <f t="shared" si="5"/>
-        <v>27.641188493103865</v>
-      </c>
-      <c r="W20" s="67">
+        <v>32.598695031689616</v>
+      </c>
+      <c r="W21" s="64">
         <f t="shared" si="5"/>
-        <v>27.60589551349965</v>
-      </c>
-      <c r="X20" s="67">
+        <v>32.521603129701276</v>
+      </c>
+      <c r="X21" s="64">
         <f t="shared" si="5"/>
-        <v>27.569214801609871</v>
-      </c>
-      <c r="Y20" s="67">
+        <v>32.444470960393318</v>
+      </c>
+      <c r="Y21" s="64">
         <f t="shared" si="5"/>
-        <v>27.531158367369663</v>
-      </c>
-      <c r="Z20" s="67">
+        <v>32.367310348545999</v>
+      </c>
+      <c r="Z21" s="64">
         <f t="shared" si="5"/>
-        <v>27.491738197205567</v>
-      </c>
-      <c r="AA20" s="67">
+        <v>32.290132171487343</v>
+      </c>
+      <c r="AA21" s="64">
         <f t="shared" si="5"/>
-        <v>27.450966253382482</v>
-      </c>
-      <c r="AB20" s="67">
+        <v>32.212946379932959</v>
+      </c>
+      <c r="AB21" s="64">
         <f t="shared" si="5"/>
-        <v>27.408854473362428</v>
-      </c>
-      <c r="AC20" s="67">
+        <v>32.135762018527103</v>
+      </c>
+      <c r="AC21" s="64">
         <f t="shared" si="5"/>
-        <v>27.365414769174986</v>
-      </c>
-      <c r="AD20" s="67">
+        <v>32.058587246088912</v>
+      </c>
+      <c r="AD21" s="64">
         <f t="shared" si="5"/>
-        <v>27.320659026799262</v>
-      </c>
-      <c r="AE20" s="67">
+        <v>31.981429355566831</v>
+      </c>
+      <c r="AE21" s="64">
         <f t="shared" si="5"/>
-        <v>27.274599105557332</v>
-      </c>
-      <c r="AF20" s="67">
+        <v>31.904294793704651</v>
+      </c>
+      <c r="AF21" s="64">
         <f t="shared" si="5"/>
-        <v>27.227246837518916</v>
-      </c>
-      <c r="AG20" s="67">
+        <v>31.827189180422515</v>
+      </c>
+      <c r="AG21" s="64">
         <f t="shared" si="5"/>
-        <v>27.178614026917153</v>
-      </c>
-      <c r="AH20" s="67">
+        <v>31.750117327916154</v>
+      </c>
+      <c r="AH21" s="64">
         <f t="shared" si="5"/>
-        <v>27.128712449575538</v>
-      </c>
-    </row>
-    <row r="21" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="63" t="s">
-        <v>326</v>
-      </c>
-      <c r="B21" s="58" t="s">
-        <v>322</v>
-      </c>
-      <c r="C21" s="62" t="s">
-        <v>329</v>
-      </c>
-      <c r="D21" s="64">
-        <f>+(D9+D10+D14)* 0.0036</f>
-        <v>15.170497668104401</v>
-      </c>
-      <c r="E21" s="64">
-        <f t="shared" ref="E21:H21" si="6">+(E9+E10+E14)* 0.0036</f>
-        <v>15.1283462930565</v>
-      </c>
-      <c r="F21" s="64">
-        <f t="shared" si="6"/>
-        <v>15.086763149119758</v>
-      </c>
-      <c r="G21" s="64">
-        <f t="shared" si="6"/>
-        <v>15.045732063612462</v>
-      </c>
-      <c r="H21" s="64">
-        <f t="shared" si="6"/>
-        <v>15.00523712257224</v>
-      </c>
-      <c r="I21" s="67">
-        <f t="shared" ref="I21:AH21" si="7">+(I9+I10+I14+I11)* 0.0036</f>
-        <v>27.96821055172137</v>
-      </c>
-      <c r="J21" s="67">
-        <f t="shared" si="7"/>
-        <v>27.952060427938289</v>
-      </c>
-      <c r="K21" s="67">
-        <f t="shared" si="7"/>
-        <v>27.934364622979814</v>
-      </c>
-      <c r="L21" s="67">
-        <f t="shared" si="7"/>
-        <v>27.915135387323247</v>
-      </c>
-      <c r="M21" s="67">
-        <f t="shared" si="7"/>
-        <v>27.89438495756859</v>
-      </c>
-      <c r="N21" s="67">
-        <f t="shared" si="7"/>
-        <v>27.872125555618592</v>
-      </c>
-      <c r="O21" s="67">
-        <f t="shared" si="7"/>
-        <v>27.848369387872459</v>
-      </c>
-      <c r="P21" s="67">
-        <f t="shared" si="7"/>
-        <v>27.823128644433229</v>
-      </c>
-      <c r="Q21" s="67">
-        <f t="shared" si="7"/>
-        <v>27.796415498328553</v>
-      </c>
-      <c r="R21" s="67">
-        <f t="shared" si="7"/>
-        <v>27.768242104744747</v>
-      </c>
-      <c r="S21" s="67">
-        <f t="shared" si="7"/>
-        <v>27.738620600274018</v>
-      </c>
-      <c r="T21" s="67">
-        <f t="shared" si="7"/>
-        <v>27.707563102174618</v>
-      </c>
-      <c r="U21" s="67">
-        <f t="shared" si="7"/>
-        <v>27.67508170764388</v>
-      </c>
-      <c r="V21" s="67">
-        <f t="shared" si="7"/>
-        <v>27.641188493103865</v>
-      </c>
-      <c r="W21" s="67">
-        <f t="shared" si="7"/>
-        <v>27.60589551349965</v>
-      </c>
-      <c r="X21" s="67">
-        <f t="shared" si="7"/>
-        <v>27.569214801609871</v>
-      </c>
-      <c r="Y21" s="67">
-        <f t="shared" si="7"/>
-        <v>27.531158367369663</v>
-      </c>
-      <c r="Z21" s="67">
-        <f t="shared" si="7"/>
-        <v>27.491738197205567</v>
-      </c>
-      <c r="AA21" s="67">
-        <f t="shared" si="7"/>
-        <v>27.450966253382482</v>
-      </c>
-      <c r="AB21" s="67">
-        <f t="shared" si="7"/>
-        <v>27.408854473362428</v>
-      </c>
-      <c r="AC21" s="67">
-        <f t="shared" si="7"/>
-        <v>27.365414769174986</v>
-      </c>
-      <c r="AD21" s="67">
-        <f t="shared" si="7"/>
-        <v>27.320659026799262</v>
-      </c>
-      <c r="AE21" s="67">
-        <f t="shared" si="7"/>
-        <v>27.274599105557332</v>
-      </c>
-      <c r="AF21" s="67">
-        <f t="shared" si="7"/>
-        <v>27.227246837518916</v>
-      </c>
-      <c r="AG21" s="67">
-        <f t="shared" si="7"/>
-        <v>27.178614026917153</v>
-      </c>
-      <c r="AH21" s="67">
-        <f t="shared" si="7"/>
-        <v>27.128712449575538</v>
-      </c>
-    </row>
-    <row r="22" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="23" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+        <v>31.673083259477465</v>
+      </c>
+    </row>
+    <row r="22" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="23" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="13" t="s">
         <v>29</v>
       </c>
@@ -14608,7 +15892,7 @@
         <v>0.99543919349214771</v>
       </c>
     </row>
-    <row r="24" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:35" x14ac:dyDescent="0.2">
       <c r="A24" s="13" t="s">
         <v>316</v>
       </c>
@@ -14743,7 +16027,7 @@
         <v>813.7431040645215</v>
       </c>
     </row>
-    <row r="25" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:35" x14ac:dyDescent="0.2">
       <c r="A25" s="13" t="s">
         <v>319</v>
       </c>
@@ -14752,133 +16036,137 @@
       </c>
       <c r="C25" s="15"/>
       <c r="D25" s="29">
-        <f t="shared" ref="D25:AH25" si="8">D11/D15</f>
+        <f t="shared" ref="D25:AH25" si="6">D11/D15</f>
         <v>0.45868652275472693</v>
       </c>
       <c r="E25" s="29">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0.4600318538182922</v>
       </c>
       <c r="F25" s="29">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0.46132678031919394</v>
       </c>
       <c r="G25" s="29">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0.46257228602861988</v>
       </c>
       <c r="H25" s="29">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0.46376932765023382</v>
       </c>
       <c r="I25" s="29">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0.46491883561769037</v>
       </c>
       <c r="J25" s="29">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0.46602171486278376</v>
       </c>
       <c r="K25" s="29">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0.46707884555542922</v>
       </c>
       <c r="L25" s="29">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0.46809108381661535</v>
       </c>
       <c r="M25" s="29">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0.46905926240541429</v>
       </c>
       <c r="N25" s="29">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0.46998419138108505</v>
       </c>
       <c r="O25" s="29">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0.47086665874125605</v>
       </c>
       <c r="P25" s="29">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0.47170743103712914</v>
       </c>
       <c r="Q25" s="29">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0.47250725396660204</v>
       </c>
       <c r="R25" s="29">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0.47326685294616455</v>
       </c>
       <c r="S25" s="29">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0.47398693366238803</v>
       </c>
       <c r="T25" s="29">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0.47466818260378374</v>
       </c>
       <c r="U25" s="29">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0.47531126757377928</v>
       </c>
       <c r="V25" s="29">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0.47591683818551811</v>
       </c>
       <c r="W25" s="29">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0.47648552633916597</v>
       </c>
       <c r="X25" s="29">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0.47701794668236613</v>
       </c>
       <c r="Y25" s="29">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0.47751469705446936</v>
       </c>
       <c r="Z25" s="29">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0.47797635891512169</v>
       </c>
       <c r="AA25" s="29">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0.47840349775778135</v>
       </c>
       <c r="AB25" s="29">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0.4787966635087007</v>
       </c>
       <c r="AC25" s="29">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0.47915639091189033</v>
       </c>
       <c r="AD25" s="29">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0.47948319990055754</v>
       </c>
       <c r="AE25" s="29">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0.47977759595548913</v>
       </c>
       <c r="AF25" s="29">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0.48004007045083213</v>
       </c>
       <c r="AG25" s="29">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0.48027110098769743</v>
       </c>
       <c r="AH25" s="29">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0.48047115171600302</v>
       </c>
+    </row>
+    <row r="29" spans="1:35" x14ac:dyDescent="0.2">
+      <c r="D29" s="67"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -15219,15 +16507,15 @@
       </c>
       <c r="B20" s="50">
         <f>Energy!D12</f>
-        <v>17122.589571324999</v>
+        <v>0</v>
       </c>
       <c r="C20" s="50">
         <f>Energy!AH12</f>
-        <v>15858.303327332134</v>
-      </c>
-      <c r="D20" s="45">
+        <v>1262.3252249727561</v>
+      </c>
+      <c r="D20" s="45" t="str">
         <f t="shared" si="0"/>
-        <v>-2.5535802827206799E-3</v>
+        <v/>
       </c>
       <c r="E20" s="46"/>
     </row>

</xml_diff>